<commit_message>
Update TdF results (tdf-results.xlsx)
</commit_message>
<xml_diff>
--- a/annual-results.xlsx
+++ b/annual-results.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M122"/>
+  <dimension ref="A1:M123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8395,6 +8395,71 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Tour de France</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Stage 6</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Tadej Pogačar</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Jonas Vingegaard</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Isaac Del Toro</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Remco Evenepoel</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Paul Seixas</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Juan Ayuso</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Florian Lipowitz</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Mattias Skjelmose</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Lenny Martinez</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>Sepp Kuss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:M20">
     <sortState ref="A2:M69">

</xml_diff>

<commit_message>
Auto-publish TdF results 2026-07-12
</commit_message>
<xml_diff>
--- a/annual-results.xlsx
+++ b/annual-results.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M125"/>
+  <dimension ref="A1:M126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8180,12 +8180,12 @@
       </c>
       <c r="K119" t="inlineStr">
         <is>
+          <t>Paul Seixas</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
           <t>Lenny Martinez</t>
-        </is>
-      </c>
-      <c r="L119" t="inlineStr">
-        <is>
-          <t>Paul Seixas</t>
         </is>
       </c>
       <c r="M119" t="inlineStr">
@@ -8235,12 +8235,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
+          <t>Florian Lipowitz</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
           <t>Lennert Van Eetvelt</t>
-        </is>
-      </c>
-      <c r="J120" t="inlineStr">
-        <is>
-          <t>Florian Lipowitz</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -8300,12 +8300,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
+          <t>Sean Quinn</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
           <t>Kévin Vauquelin</t>
-        </is>
-      </c>
-      <c r="J121" t="inlineStr">
-        <is>
-          <t>Sean Quinn</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -8495,22 +8495,22 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
+          <t>Phil Bauhaus</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
           <t>Huub Artz</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr">
-        <is>
-          <t>Phil Bauhaus</t>
-        </is>
-      </c>
       <c r="K124" t="inlineStr">
         <is>
+          <t>Mads Pedersen</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
           <t>Dorian Godon</t>
-        </is>
-      </c>
-      <c r="L124" t="inlineStr">
-        <is>
-          <t>Mads Pedersen</t>
         </is>
       </c>
       <c r="M124" t="inlineStr">
@@ -8581,6 +8581,71 @@
       <c r="M125" t="inlineStr">
         <is>
           <t>Milan Fretin</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>46215</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Tour de France</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Stage 9</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Mathieu Van Der Poel</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Tobias Halland Johannessen</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Tom Pidcock</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Alex Baudin</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Filippo Ganna</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Mads Pedersen</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Michael Matthews</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Jordan Jegat</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>Nicolas Breuillard</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>Sean Quinn</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish TdF results 2026-07-17
</commit_message>
<xml_diff>
--- a/annual-results.xlsx
+++ b/annual-results.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M129"/>
+  <dimension ref="A1:M130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8594,7 +8594,7 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="n">
+      <c r="A126" t="n">
         <v>46215</v>
       </c>
       <c r="B126" t="inlineStr">
@@ -8789,7 +8789,7 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" t="n">
+      <c r="A129" s="2" t="n">
         <v>46219</v>
       </c>
       <c r="B129" t="inlineStr">
@@ -8850,6 +8850,71 @@
       <c r="M129" t="inlineStr">
         <is>
           <t>Huub Artz</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Tour de France</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Stage 13</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Mauro Schmid</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Harold Tejada</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Tom Pidcock</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Maxim Van Gils</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Brandon Mcnulty</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Jordan Jegat</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Kévin Vauquelin</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Clement Braz Afonso</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>Tim Wellens</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>Luke Plapp</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-publish TdF results 2026-07-18
</commit_message>
<xml_diff>
--- a/annual-results.xlsx
+++ b/annual-results.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M130"/>
+  <dimension ref="A1:M131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -8918,6 +8918,71 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>46221</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Tour de France</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Stage 14</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Tadej Pogačar</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Isaac Del Toro</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Paul Seixas</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Jonas Vingegaard</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Remco Evenepoel</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Florian Lipowitz</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Juan Ayuso</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Richard Carapaz</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>Tobias Halland Johannessen</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>Mattias Skjelmose</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:M20">
     <sortState ref="A2:M69">

</xml_diff>

<commit_message>
Auto-publish TdF results 2026-07-25
</commit_message>
<xml_diff>
--- a/annual-results.xlsx
+++ b/annual-results.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M136"/>
+  <dimension ref="A1:M137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17.85546875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9304,6 +9304,71 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>46228</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Tour de France</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Stage 20</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Richard Carapaz</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Remco Evenepoel</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Sepp Kuss</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Tadej Pogačar</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Isaac Del Toro</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Jai Hindley</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Lenny Martinez</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Mattias Skjelmose</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>Juan Ayuso</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>Paul Seixas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:M20">
     <sortState ref="A2:M69">

</xml_diff>